<commit_message>
feat: cushion items routed to line 9 + set group key overrides order name
</commit_message>
<xml_diff>
--- a/품목마스터/마감작업자별 생산가능품목_코드목록_v2.xlsx
+++ b/품목마스터/마감작업자별 생산가능품목_코드목록_v2.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16440" windowHeight="8655" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16440" windowHeight="8655" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -17,13 +17,14 @@
     <sheet name="품목군별코드" sheetId="4" r:id="rId3"/>
     <sheet name="품목군코드상세" sheetId="5" r:id="rId4"/>
     <sheet name="특정라인 지정" sheetId="6" r:id="rId5"/>
+    <sheet name="셋트구분" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2770" uniqueCount="1095">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2837" uniqueCount="1108">
   <si>
     <t>마감작업자 생산가능품목</t>
   </si>
@@ -3308,6 +3309,49 @@
   </si>
   <si>
     <t>홀리데이 미니 터미널 (좌) 커버+내장재 ASSY</t>
+  </si>
+  <si>
+    <t>L849L</t>
+  </si>
+  <si>
+    <t>HCS8812R</t>
+  </si>
+  <si>
+    <t>HCS8812L</t>
+  </si>
+  <si>
+    <t>L846</t>
+  </si>
+  <si>
+    <t>L841L</t>
+  </si>
+  <si>
+    <t>L845</t>
+  </si>
+  <si>
+    <t>밴쿠버 3인 몸통(가죽)</t>
+  </si>
+  <si>
+    <t>HCS8813L</t>
+  </si>
+  <si>
+    <t>HCS8811R</t>
+  </si>
+  <si>
+    <t>품목명칭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>색상</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>품목코드</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>셋트 구분</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -3435,7 +3479,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -3469,6 +3513,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -15915,4 +15962,330 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" style="13"/>
+    <col min="2" max="2" width="18.125" style="13" customWidth="1"/>
+    <col min="3" max="3" width="12" style="13" customWidth="1"/>
+    <col min="4" max="4" width="25.375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>1105</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="13">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="13">
+        <v>1</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="13">
+        <v>2</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="13">
+        <v>2</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="13">
+        <v>3</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>1100</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="13">
+        <v>3</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>1100</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
+        <v>4</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <v>4</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="13">
+        <v>5</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="13">
+        <v>6</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
+        <v>7</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="13">
+        <v>8</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="13">
+        <v>9</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>1100</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="13">
+        <v>10</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
+        <v>11</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <v>12</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="13">
+        <v>12</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="13">
+        <v>13</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="13">
+        <v>13</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="13">
+        <v>14</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
+        <v>14</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>357</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add 셋트 15·16 for RAXXZ002·RAXXZ003 (저품질 사티 1인 좌/우)
</commit_message>
<xml_diff>
--- a/품목마스터/마감작업자별 생산가능품목_코드목록_v2.xlsx
+++ b/품목마스터/마감작업자별 생산가능품목_코드목록_v2.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16440" windowHeight="8655" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16440" windowHeight="8655" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2564" uniqueCount="1068">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2576" uniqueCount="1074">
   <si>
     <t>마감작업자 생산가능품목</t>
   </si>
@@ -3241,6 +3241,29 @@
   </si>
   <si>
     <t>폴디</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RAXXZ003</t>
+  </si>
+  <si>
+    <t>L735</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[저품질] 사티 1인 (우)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[저품질] 사티 1인 (좌)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RAXXZ002</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>L730</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3369,7 +3392,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -3407,6 +3430,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -14809,13 +14835,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="13"/>
     <col min="2" max="2" width="18.125" style="13" customWidth="1"/>
     <col min="3" max="3" width="12" style="13" customWidth="1"/>
-    <col min="4" max="4" width="25.375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.625" style="13" customWidth="1"/>
     <col min="5" max="16384" width="9" style="13"/>
   </cols>
   <sheetData>
@@ -14861,43 +14887,71 @@
         <v>315</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="13">
+        <v>2</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>313</v>
+      </c>
+    </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <v>2</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>1052</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B6" s="13" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="13">
+        <v>3</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>1056</v>
       </c>
-      <c r="C6" s="13" t="s">
-        <v>1052</v>
-      </c>
-      <c r="D6" s="13" t="s">
+      <c r="C7" s="13" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>1057</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>1054</v>
+        <v>1049</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>313</v>
@@ -14905,226 +14959,254 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>1056</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>1054</v>
+        <v>1049</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>315</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="13">
+        <v>5</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>1055</v>
+      </c>
+    </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>1057</v>
+        <v>305</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>1049</v>
+        <v>1052</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>313</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>1056</v>
+        <v>305</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>1049</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>315</v>
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="13">
+        <v>8</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="13">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>1055</v>
+        <v>317</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="13">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>1052</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>1055</v>
+        <v>317</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="13">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>1049</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>1055</v>
+        <v>317</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="13">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>300</v>
+        <v>1051</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>1053</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="13">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>300</v>
+        <v>1050</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="13">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>300</v>
+        <v>1051</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>1052</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="13">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>300</v>
+        <v>1050</v>
       </c>
       <c r="C20" s="13" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="13">
+        <v>14</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C21" s="13" t="s">
         <v>1049</v>
       </c>
-      <c r="D20" s="13" t="s">
-        <v>317</v>
+      <c r="D21" s="13" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="13">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="13">
-        <v>12</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>1050</v>
+        <v>15</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>1068</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>1053</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>311</v>
+        <v>1069</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="13">
+        <v>15</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>1071</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="13">
-        <v>13</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>1051</v>
+        <v>16</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>1068</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>1052</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>309</v>
+        <v>1073</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>1070</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="13">
-        <v>13</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>1050</v>
+        <v>16</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>1072</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>1052</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="13">
-        <v>14</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>1051</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>1049</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="13">
-        <v>14</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>1050</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>1049</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>311</v>
+        <v>1073</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>1071</v>
       </c>
     </row>
   </sheetData>

</xml_diff>